<commit_message>
Sync latest charts and notebook
</commit_message>
<xml_diff>
--- a/data/raw/умное_потребление_данные.xlsx
+++ b/data/raw/умное_потребление_данные.xlsx
@@ -23,6 +23,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STM_Топ_Категорий" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STM_Мотивация" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosstat_Оборот_Розницы" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSE_Сбережения_Кредиты" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSE_Защита_Прав" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSE_Портрет_Потребителя" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSE_Макро_Контекст" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chizhik_ВШЭ_Индекс" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chizhik_ВШЭ_Сегменты" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chizhik_ВШЭ_Паттерны" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosstat_Структура_Расходов" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosstat_Интернет_Торговля" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2765,6 +2774,633 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>wave</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>есть_ликвидные_сбережения_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>есть_непогашенный_кредит_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>нет_сбережений_нет_кредитов_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>только_сбережения_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>только_кредит_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>сбережения_и_кредит_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: НИУ ВШЭ, Барометр экономического поведения домохозяйств №2-2026, опрос ЭПДХ (7 волн, 2023-2025), репрезентативная выборка 55 регионов РФ, 6000-6800 респондентов на волну. Ключевой показатель для темы: доля без сбережений и без кредитов ('живут на текущие доходы') выросла с 41,4% до 53,3% — прямой индикатор вынужденной финансовой осторожности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Июнь-июль 2023</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Сентябрь-ноябрь 2023</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Декабрь2023-Февраль2024</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Апрель-май 2024</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Октябрь-ноябрь 2024</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Апрель-май 2025</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Октябрь-ноябрь 2025</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I1:I7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>wave</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>покупали_некачественные_товары_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>из_них_предпринимали_действия_по_защите_прав_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Дополнительные данные (не по волнам, усреднённо за 2023-2025):</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>value_pct</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Среднее по волнам: покупали некачественный товар/услугу</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Предъявляли претензию продавцу/производителю</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Обращались в организации по защите прав потребителей</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Доводили дело до суда</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2025 весна</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2025 осень</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>23.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>группа</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>характеристика</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>направление</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: НИУ ВШЭ, Барометр №2-2026, раздел 4, статистический анализ скорректированных стандартизированных остатков по данным ЭПДХ 1-7 волн.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>25-34 года</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>чаще покупают некачественные товары (уязвимая группа)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>65+ лет</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>реже сталкиваются с некачественными товарами</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Место жительства</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>города 100 тыс.-1 млн чел.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>чаще сталкиваются с некачественными товарами</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Место жительства</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>сельская местность</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>реже сталкиваются с некачественными товарами</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Доход</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>низкий (едва сводят концы с концами)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>чаще покупают некачественные товары (уязвимая группа)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Состав семьи</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>есть дети до 16 лет</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>чаще сталкиваются с некачественными товарами</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Пол</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>мужчины</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>чаще отстаивают права</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Образование</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>высшее</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>чаще отстаивают права</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>18-44 года</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>более активны в защите прав</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>65+ лет</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>заметно реже отстаивают права</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Доход</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>финансово необеспеченные не ограничены</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>чаще отстаивают права</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Канал покупки</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>покупают онлайн</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>чаще отстаивают права, чем офлайн-покупатели</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:D12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3159,6 +3795,2494 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: НИУ ВШЭ, Барометр экономического поведения домохозяйств №2-2026 (данные Росстата, Банка России, ЭПДХ ВШЭ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Рост реальных располагаемых денежных доходов, г/г</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Среднедушевой денежный доход (номинал)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>69000</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>руб./мес</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Среднедушевой доход, среднее за год</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>75000</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>руб./мес</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Медианный доход</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>руб./мес</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Коэффициент фондов</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>раз</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Коэффициент фондов</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>раз</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Коэффициент Джини</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0.422</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>индекс</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Коэффициент Джини</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>индекс</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Рост реальной зарплаты, г/г</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Рост реальной зарплаты, г/г</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>декабрь 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Средняя зарплата (номинал)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>112700</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>руб./мес</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>март 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Средняя пенсия (номинал)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>25400</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>руб./мес</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>апрель 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Ставка НДС (базовая)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>с 1 января 2026 (было 20%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Рост расходов домохозяйств от повышения НДС (оценка)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>2026, оценка НИУ ВШЭ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Влияние повышения НДС на цены (оценка Банка России)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>п.п.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>январь 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Доля домохозяйств с ипотекой</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>устойчиво, 2023-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Средний ежемесячный платёж по ипотеке</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>26000</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>руб./ДХ</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Доля домохозяйств, арендующих жильё</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>устойчиво, 2023-2025</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F1:F10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>value_2024</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>value_2025</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: НИУ ВШЭ + 'Чижик' (X5), опрос &gt;6000 респондентов 18+, 2025 г., сопоставлено с волной 2024 г.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Доля умных потребителей (совокупный индекс)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Индекс умного потребления (п.п.)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>п.п.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ориентируются на приемлемое качество</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Ориентируются исключительно на низкую цену</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Не готовы переплачивать за известный бренд</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Планируют покупки заранее</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Легко ориентируются среди множества предложений</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Стремятся минимизировать время на покупки</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F1:F8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>smart_consumption_share_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: НИУ ВШЭ + 'Чижик' (X5), 2025 (часть показателей — объединённые данные 2024-2025). Пустая ячейка = показатель не публиковался для этой волны.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Семейное положение</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Не состоят в браке</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Семейное положение</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Состоят в браке</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Наличие детей</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Нет детей</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Наличие детей</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Есть дети</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Пол</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Мужчины</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Пол</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Женщины</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Возраст</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Города-миллионники</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Города-миллионники</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Города 100 тыс.-1 млн</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Города 100 тыс.-1 млн</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Небольшие города</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Небольшие города</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Сельская местность</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Тип населённого пункта</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Сельская местность</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Импульсивность покупок</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Не склонны к импульсивным покупкам</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Импульсивность покупок</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Склонны к импульсивным покупкам</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Покупка новинок</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Реже покупают новинки</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Покупка новинок</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Чаще покупают новинки</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Участие в распродажах</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Реже участвуют в распродажах</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Участие в распродажах</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Чаще участвуют в распродажах</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Канал покупки</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Офлайн-шопинг</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Канал покупки</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Онлайн-шопинг</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:E30"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>group_pair</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>value_group1</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>value_group2</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Столбцы value_group1/value_group2 соответствуют первой/второй группе из group_pair (%). Источник: НИУ ВШЭ + 'Чижик', 2024-2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>В браке vs Одинокие</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Ориентируются только на низкую цену</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>В браке vs Одинокие</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Ориентируются на приемлемое качество</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Есть дети vs Нет детей</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Ориентируются только на низкую цену</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Женщины vs Мужчины</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Решение о покупке сразу при приемлемом качестве</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Женщины vs Мужчины</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Не готовы переплачивать за бренд</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Женщины vs Мужчины</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Планируют покупки заранее</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Женщины vs Мужчины</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Стремятся минимизировать время на покупки</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:E7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>group_type</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>spend_per_member_rub</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>food_share_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>nonfood_share_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>alcohol_share_pct</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>services_share_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: Росстат, 'Торговля в России. 2025', табл. 2.45 (выборочное обследование бюджетов ДХ). food/nonfood/alcohol/services_share_pct — доли от общего объёма расходов на конечное потребление. Приведены не все строки оригинала (полный разрез по годам доступен в PDF на стр. 56-57 при необходимости).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Все ДХ</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Все домашние хозяйства</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>21154.3</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>26.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>1 человек</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>33236.8</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>2 человека</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>24377.6</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>3 человека</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>21988.7</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>4 человека</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>17796.4</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>5 и более человек</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>13596.9</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>1-я (наименьшие ресурсы)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>8389.5</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>2-я</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>12850.9</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>3-я</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>17122.1</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>4-я</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>23643.4</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>26.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>5-я (наибольшие ресурсы)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>43768.8</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Все ДХ</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Все домашние хозяйства</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>23787.9</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>26.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>1 человек</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>40779</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>26.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>5 и более человек</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>15175.4</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>21.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>1-я (наименьшие ресурсы)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>9577.6</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>22.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>5-я (наибольшие ресурсы)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>49760.8</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Все ДХ</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Все домашние хозяйства</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>26881</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>26.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>1 человек</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>42067.2</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>По составу</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>5 и более человек</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>15692.9</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>24.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>1-я (наименьшие ресурсы)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>10615.5</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>22.8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>По доходу (20% группы)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>5-я (наибольшие ресурсы)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>57201.4</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>29.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I1:I21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Источник: Росстат, 'Торговля в России. 2025', табл. 2.17-2.20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Доля товаров, проданных через интернет</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Доля товаров, проданных через интернет</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Доля товаров, проданных через интернет</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Доля товаров, проданных через интернет</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Доля товаров, проданных через интернет</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Заказов через маркетплейсы, млн</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3726.5</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>млн заказов</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Заказов через маркетплейсы, млн</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5588.4</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>млн заказов</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Брендированных ПВЗ маркетплейсов</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>136581</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Брендированных ПВЗ маркетплейсов</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>229321</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Лица 15+, пользующиеся интернетом для покупок</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Лица 15+, пользующиеся интернетом для покупок</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Из них: постоянно покупают продукты питания/гигиену онлайн</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Из них: постоянно покупают продукты питания/гигиену онлайн</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Из них: постоянно покупают одежду/обувь онлайн</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Из них: постоянно покупают одежду/обувь онлайн</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:E15"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>